<commit_message>
Study capabilities in English: English prompts, keywords and plan contents
- All AI prompts (Project instructions, split into parts, study session,
  review, dataset description) are now in English and ask the tutor to teach
  only in English, define new terms, and flag up to two English mistakes
- Review card gains KEY TERMS; verdicts are REVIEW DONE / REVIEW AGAIN
- Import accepts English keywords (CAPABILITY, PROJECT, SOURCES, DEPTH,
  SESSIONS, DEADLINE, STATUS: On hold, AREA) in text and JSON
- partes.txt renamed to parts.txt
- Capabilities plan and import file use English names, sources and milestones
- Update templates, README and study method guide

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JeoC1T6GvSfXrBZdTVZHj4
</commit_message>
<xml_diff>
--- a/planejamento/plano-capacidades.xlsx
+++ b/planejamento/plano-capacidades.xlsx
@@ -22,8 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -129,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,10 +146,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -160,10 +161,10 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -175,10 +176,10 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -190,10 +191,10 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -205,7 +206,7 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -215,7 +216,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,64 +224,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -780,7 +736,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Estatística para DS</t>
+          <t>Statistics for Data Science</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -799,25 +755,25 @@
       <c r="F5" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="G5" s="40" t="n">
+      <c r="G5" s="7" t="n">
         <v>46296</v>
       </c>
       <c r="H5" s="4">
         <f>ROUNDUP(E5*IF(D5="Profundo",Premissas!$B$4,Premissas!$B$5)/F5,0)</f>
         <v/>
       </c>
-      <c r="I5" s="41">
+      <c r="I5" s="8">
         <f>G5+H5*7</f>
         <v/>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Livro: Practical Statistics for Data Scientists, 2ª ed. (Bruce, Bruce &amp; Gedeck)</t>
+          <t>Book: Practical Statistics for Data Scientists, 2nd ed. (Bruce, Bruce &amp; Gedeck)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Livro: Estatística Básica (Morettin &amp; Bussab)</t>
+          <t>Book: OpenIntro Statistics, 4th ed. (Diez, Çetinkaya-Rundel &amp; Barr), free at openintro.org</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
@@ -839,7 +795,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Lógica de programação e bibliotecas Python para DS</t>
+          <t>Programming Logic and Python Libraries for Data Science</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -858,25 +814,25 @@
       <c r="F6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="40" t="n">
+      <c r="G6" s="7" t="n">
         <v>46296</v>
       </c>
       <c r="H6" s="4">
         <f>ROUNDUP(E6*IF(D6="Profundo",Premissas!$B$4,Premissas!$B$5)/F6,0)</f>
         <v/>
       </c>
-      <c r="I6" s="41">
+      <c r="I6" s="8">
         <f>G6+H6*7</f>
         <v/>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Livro: Python for Data Analysis, 3ª ed. (Wes McKinney), grátis em wesmckinney.com/book</t>
+          <t>Book: Python for Data Analysis, 3rd ed. (Wes McKinney), free at wesmckinney.com/book</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Repositório: github.com/jakevdp/PythonDataScienceHandbook</t>
+          <t>Repository: github.com/jakevdp/PythonDataScienceHandbook</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -898,7 +854,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>SQL / modelagem de dados</t>
+          <t>SQL / Data Modeling</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -917,25 +873,25 @@
       <c r="F7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="40" t="n">
+      <c r="G7" s="7" t="n">
         <v>46296</v>
       </c>
       <c r="H7" s="4">
         <f>ROUNDUP(E7*IF(D7="Profundo",Premissas!$B$4,Premissas!$B$5)/F7,0)</f>
         <v/>
       </c>
-      <c r="I7" s="41">
+      <c r="I7" s="8">
         <f>G7+H7*7</f>
         <v/>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Livro: Learning SQL, 3ª ed. (Alan Beaulieu)</t>
+          <t>Book: Learning SQL, 3rd ed. (Alan Beaulieu)</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>Livro: The Data Warehouse Toolkit, 3ª ed. (Kimball &amp; Ross)</t>
+          <t>Book: The Data Warehouse Toolkit, 3rd ed. (Kimball &amp; Ross)</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
@@ -957,7 +913,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Git conceitual</t>
+          <t>Git (Conceptual)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -976,20 +932,20 @@
       <c r="F8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G8" s="40" t="n">
+      <c r="G8" s="7" t="n">
         <v>46296</v>
       </c>
       <c r="H8" s="4">
         <f>ROUNDUP(E8*IF(D8="Profundo",Premissas!$B$4,Premissas!$B$5)/F8,0)</f>
         <v/>
       </c>
-      <c r="I8" s="41">
+      <c r="I8" s="8">
         <f>G8+H8*7</f>
         <v/>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Livro: Pro Git, 2ª ed. (Chacon &amp; Straub), grátis em git-scm.com/book — capítulos 1–3 e 10</t>
+          <t>Book: Pro Git, 2nd ed. (Chacon &amp; Straub), free at git-scm.com/book — chapters 1–3 and 10</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1016,7 +972,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Engenharia de prompt / harness / spec</t>
+          <t>Prompt Engineering / Harness / Spec</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -1035,25 +991,25 @@
       <c r="F9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="40" t="n">
+      <c r="G9" s="7" t="n">
         <v>46332</v>
       </c>
       <c r="H9" s="4">
         <f>ROUNDUP(E9*IF(D9="Profundo",Premissas!$B$4,Premissas!$B$5)/F9,0)</f>
         <v/>
       </c>
-      <c r="I9" s="41">
+      <c r="I9" s="8">
         <f>G9+H9*7</f>
         <v/>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Repositório: github.com/anthropics/prompt-eng-interactive-tutorial</t>
+          <t>Repository: github.com/anthropics/prompt-eng-interactive-tutorial</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Artigo: Building effective agents (Anthropic); documentação da Anthropic sobre prompts e agentes</t>
+          <t>Article: Building effective agents (Anthropic); Docs: Anthropic documentation on prompting and agents</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
@@ -1075,7 +1031,7 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Matemática para DS</t>
+          <t>Mathematics for Data Science</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -1094,30 +1050,30 @@
       <c r="F10" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G10" s="42" t="n">
+      <c r="G10" s="12" t="n">
         <v>46391</v>
       </c>
       <c r="H10" s="9">
         <f>ROUNDUP(E10*IF(D10="Profundo",Premissas!$B$4,Premissas!$B$5)/F10,0)</f>
         <v/>
       </c>
-      <c r="I10" s="43">
+      <c r="I10" s="13">
         <f>G10+H10*7</f>
         <v/>
       </c>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>Livro: Mathematics for Machine Learning (Deisenroth, Faisal &amp; Ong), grátis em mml-book.github.io</t>
+          <t>Book: Mathematics for Machine Learning (Deisenroth, Faisal &amp; Ong), free at mml-book.github.io</t>
         </is>
       </c>
       <c r="K10" s="10" t="inlineStr">
         <is>
-          <t>Curso: Essence of Linear Algebra (3Blue1Brown)</t>
+          <t>Course: Essence of Linear Algebra (3Blue1Brown)</t>
         </is>
       </c>
       <c r="L10" s="10" t="inlineStr">
         <is>
-          <t>Estatística para DS</t>
+          <t>Statistics for Data Science</t>
         </is>
       </c>
       <c r="M10" s="10" t="inlineStr">
@@ -1134,7 +1090,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>EDA avançada</t>
+          <t>Advanced EDA</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -1153,30 +1109,30 @@
       <c r="F11" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="G11" s="42" t="n">
+      <c r="G11" s="12" t="n">
         <v>46391</v>
       </c>
       <c r="H11" s="9">
         <f>ROUNDUP(E11*IF(D11="Profundo",Premissas!$B$4,Premissas!$B$5)/F11,0)</f>
         <v/>
       </c>
-      <c r="I11" s="43">
+      <c r="I11" s="13">
         <f>G11+H11*7</f>
         <v/>
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>Livro: Feature Engineering and Selection (Kuhn &amp; Johnson), grátis em feat.engineering</t>
+          <t>Book: Feature Engineering and Selection (Kuhn &amp; Johnson), free at feat.engineering</t>
         </is>
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>Repositório: github.com/jakevdp/PythonDataScienceHandbook; as suas bases</t>
+          <t>Repository: github.com/jakevdp/PythonDataScienceHandbook; My own datasets</t>
         </is>
       </c>
       <c r="L11" s="10" t="inlineStr">
         <is>
-          <t>Estatística; Python para DS</t>
+          <t>Statistics; Python for Data Science</t>
         </is>
       </c>
       <c r="M11" s="10" t="inlineStr">
@@ -1193,7 +1149,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Visualização de dados</t>
+          <t>Data Visualization</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -1212,30 +1168,30 @@
       <c r="F12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="42" t="n">
+      <c r="G12" s="12" t="n">
         <v>46391</v>
       </c>
       <c r="H12" s="9">
         <f>ROUNDUP(E12*IF(D12="Profundo",Premissas!$B$4,Premissas!$B$5)/F12,0)</f>
         <v/>
       </c>
-      <c r="I12" s="43">
+      <c r="I12" s="13">
         <f>G12+H12*7</f>
         <v/>
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>Livro: Fundamentals of Data Visualization (Claus Wilke), grátis em clauswilke.com/dataviz</t>
+          <t>Book: Fundamentals of Data Visualization (Claus Wilke), free at clauswilke.com/dataviz</t>
         </is>
       </c>
       <c r="K12" s="10" t="inlineStr">
         <is>
-          <t>Documentação: matplotlib e seaborn</t>
+          <t>Docs: matplotlib and seaborn</t>
         </is>
       </c>
       <c r="L12" s="10" t="inlineStr">
         <is>
-          <t>Python para DS</t>
+          <t>Python for Data Science</t>
         </is>
       </c>
       <c r="M12" s="10" t="inlineStr">
@@ -1252,7 +1208,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Storytelling</t>
+          <t>Data Storytelling</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -1271,30 +1227,30 @@
       <c r="F13" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G13" s="42" t="n">
+      <c r="G13" s="12" t="n">
         <v>46447</v>
       </c>
       <c r="H13" s="9">
         <f>ROUNDUP(E13*IF(D13="Profundo",Premissas!$B$4,Premissas!$B$5)/F13,0)</f>
         <v/>
       </c>
-      <c r="I13" s="43">
+      <c r="I13" s="13">
         <f>G13+H13*7</f>
         <v/>
       </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>Livro: Storytelling with Data (Cole Nussbaumer Knaflic)</t>
+          <t>Book: Storytelling with Data (Cole Nussbaumer Knaflic)</t>
         </is>
       </c>
       <c r="K13" s="10" t="inlineStr">
         <is>
-          <t>Livro: Storytelling with Data: Let's Practice! (Knaflic)</t>
+          <t>Book: Storytelling with Data: Let's Practice! (Knaflic)</t>
         </is>
       </c>
       <c r="L13" s="10" t="inlineStr">
         <is>
-          <t>Visualização de dados</t>
+          <t>Data Visualization</t>
         </is>
       </c>
       <c r="M13" s="10" t="inlineStr">
@@ -1311,7 +1267,7 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Engenharia de IA</t>
+          <t>AI Engineering</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -1330,30 +1286,30 @@
       <c r="F14" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="G14" s="44" t="n">
+      <c r="G14" s="17" t="n">
         <v>46482</v>
       </c>
       <c r="H14" s="14">
         <f>ROUNDUP(E14*IF(D14="Profundo",Premissas!$B$4,Premissas!$B$5)/F14,0)</f>
         <v/>
       </c>
-      <c r="I14" s="45">
+      <c r="I14" s="18">
         <f>G14+H14*7</f>
         <v/>
       </c>
       <c r="J14" s="15" t="inlineStr">
         <is>
-          <t>Livro: AI Engineering (Chip Huyen)</t>
+          <t>Book: AI Engineering (Chip Huyen)</t>
         </is>
       </c>
       <c r="K14" s="15" t="inlineStr">
         <is>
-          <t>Artigo: Building effective agents (Anthropic)</t>
+          <t>Article: Building effective agents (Anthropic)</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
         <is>
-          <t>Prompt / harness / spec; Python</t>
+          <t>Prompt Engineering / Harness / Spec; Python</t>
         </is>
       </c>
       <c r="M14" s="15" t="inlineStr">
@@ -1370,7 +1326,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>Engenharia de dados e governança</t>
+          <t>Data Engineering and Governance</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
@@ -1389,30 +1345,30 @@
       <c r="F15" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="G15" s="44" t="n">
+      <c r="G15" s="17" t="n">
         <v>46482</v>
       </c>
       <c r="H15" s="14">
         <f>ROUNDUP(E15*IF(D15="Profundo",Premissas!$B$4,Premissas!$B$5)/F15,0)</f>
         <v/>
       </c>
-      <c r="I15" s="45">
+      <c r="I15" s="18">
         <f>G15+H15*7</f>
         <v/>
       </c>
       <c r="J15" s="15" t="inlineStr">
         <is>
-          <t>Livro: Fundamentals of Data Engineering (Reis &amp; Housley)</t>
+          <t>Book: Fundamentals of Data Engineering (Reis &amp; Housley)</t>
         </is>
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>Repositório: github.com/DataTalksClub/data-engineering-zoomcamp; Livro: Data Governance: The Definitive Guide (Eryurek et al.)</t>
+          <t>Repository: github.com/DataTalksClub/data-engineering-zoomcamp; Book: Data Governance: The Definitive Guide (Eryurek et al.)</t>
         </is>
       </c>
       <c r="L15" s="15" t="inlineStr">
         <is>
-          <t>SQL / modelagem; Python</t>
+          <t>SQL / Data Modeling; Python</t>
         </is>
       </c>
       <c r="M15" s="15" t="inlineStr">
@@ -1429,7 +1385,7 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Ciência da computação</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
@@ -1448,30 +1404,30 @@
       <c r="F16" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="G16" s="44" t="n">
+      <c r="G16" s="17" t="n">
         <v>46482</v>
       </c>
       <c r="H16" s="14">
         <f>ROUNDUP(E16*IF(D16="Profundo",Premissas!$B$4,Premissas!$B$5)/F16,0)</f>
         <v/>
       </c>
-      <c r="I16" s="45">
+      <c r="I16" s="18">
         <f>G16+H16*7</f>
         <v/>
       </c>
       <c r="J16" s="15" t="inlineStr">
         <is>
-          <t>Livro: Grokking Algorithms, 2ª ed. (Aditya Bhargava)</t>
+          <t>Book: Grokking Algorithms, 2nd ed. (Aditya Bhargava)</t>
         </is>
       </c>
       <c r="K16" s="15" t="inlineStr">
         <is>
-          <t>Curso: CS50x (Harvard, gratuito)</t>
+          <t>Course: CS50x (Harvard, free)</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
         <is>
-          <t>Lógica de programação</t>
+          <t>Programming Logic</t>
         </is>
       </c>
       <c r="M16" s="15" t="inlineStr">
@@ -1488,7 +1444,7 @@
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>Engenharia de ML</t>
+          <t>ML Engineering</t>
         </is>
       </c>
       <c r="C17" s="20" t="inlineStr">
@@ -1507,30 +1463,30 @@
       <c r="F17" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="G17" s="46" t="n">
+      <c r="G17" s="22" t="n">
         <v>46573</v>
       </c>
       <c r="H17" s="19">
         <f>ROUNDUP(E17*IF(D17="Profundo",Premissas!$B$4,Premissas!$B$5)/F17,0)</f>
         <v/>
       </c>
-      <c r="I17" s="47">
+      <c r="I17" s="23">
         <f>G17+H17*7</f>
         <v/>
       </c>
       <c r="J17" s="20" t="inlineStr">
         <is>
-          <t>Livro: Designing Machine Learning Systems (Chip Huyen)</t>
+          <t>Book: Designing Machine Learning Systems (Chip Huyen)</t>
         </is>
       </c>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Repositório: github.com/GokuMohandas/Made-With-ML; Livro: Hands-On Machine Learning (Aurélien Géron)</t>
+          <t>Repository: github.com/GokuMohandas/Made-With-ML; Book: Hands-On Machine Learning (Aurélien Géron)</t>
         </is>
       </c>
       <c r="L17" s="20" t="inlineStr">
         <is>
-          <t>Matemática; Estatística; EDA</t>
+          <t>Mathematics; Statistics; Advanced EDA</t>
         </is>
       </c>
       <c r="M17" s="20" t="inlineStr">
@@ -1547,7 +1503,7 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>System design</t>
+          <t>System Design</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
@@ -1566,30 +1522,30 @@
       <c r="F18" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="G18" s="46" t="n">
+      <c r="G18" s="22" t="n">
         <v>46573</v>
       </c>
       <c r="H18" s="19">
         <f>ROUNDUP(E18*IF(D18="Profundo",Premissas!$B$4,Premissas!$B$5)/F18,0)</f>
         <v/>
       </c>
-      <c r="I18" s="47">
+      <c r="I18" s="23">
         <f>G18+H18*7</f>
         <v/>
       </c>
       <c r="J18" s="20" t="inlineStr">
         <is>
-          <t>Livro: Designing Data-Intensive Applications (Martin Kleppmann)</t>
+          <t>Book: Designing Data-Intensive Applications (Martin Kleppmann)</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>Repositório: github.com/donnemartin/system-design-primer</t>
+          <t>Repository: github.com/donnemartin/system-design-primer</t>
         </is>
       </c>
       <c r="L18" s="20" t="inlineStr">
         <is>
-          <t>Engenharia de dados; Engenharia de IA</t>
+          <t>Data Engineering; AI Engineering</t>
         </is>
       </c>
       <c r="M18" s="20" t="inlineStr">
@@ -1606,7 +1562,7 @@
       </c>
       <c r="B19" s="25" t="inlineStr">
         <is>
-          <t>Inglês</t>
+          <t>English</t>
         </is>
       </c>
       <c r="C19" s="25" t="inlineStr">
@@ -1625,23 +1581,23 @@
       <c r="F19" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="48" t="n">
+      <c r="G19" s="27" t="n">
         <v>46296</v>
       </c>
       <c r="H19" s="26" t="n">
         <v>52</v>
       </c>
-      <c r="I19" s="48" t="n">
+      <c r="I19" s="27" t="n">
         <v>46660</v>
       </c>
       <c r="J19" s="25" t="inlineStr">
         <is>
-          <t>Livro: English Grammar in Use (Raymond Murphy) — só para os tópicos de gramática</t>
+          <t>Book: English Grammar in Use (Raymond Murphy) — grammar topics only</t>
         </is>
       </c>
       <c r="K19" s="25" t="inlineStr">
         <is>
-          <t>Palestras técnicas (PyData, conferências) e as fontes em inglês das outras capacidades</t>
+          <t>Tech talks (PyData, conferences); The sources of every other capability, all studied in English</t>
         </is>
       </c>
       <c r="L19" s="25" t="inlineStr">
@@ -1651,14 +1607,14 @@
       </c>
       <c r="M19" s="25" t="inlineStr">
         <is>
-          <t>Habilidade, não conceito: 12 marcos mensais (aba Inglês — marcos) + hábito diário no almoço.</t>
+          <t>Habilidade, não conceito: 12 marcos mensais (aba Inglês — marcos) + hábito diário no almoço + todas as capacidades estudadas em inglês (imersão diária).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Fontes: sugestões para quando você ainda não tiver material; troque à vontade. A primeira fonte é a que define a ordem das partes.</t>
+          <t>Fontes: sugestões em inglês (o estudo das capacidades é em inglês); troque à vontade. A primeira fonte é a que define a ordem das partes.</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1729,7 @@
           <t>Início da onda 1</t>
         </is>
       </c>
-      <c r="B8" s="49" t="n">
+      <c r="B8" s="31" t="n">
         <v>46296</v>
       </c>
       <c r="C8" s="29" t="inlineStr">
@@ -2118,7 +2074,7 @@
       </c>
       <c r="E12" s="29" t="inlineStr">
         <is>
-          <t>Projetos / Inglês</t>
+          <t>Projetos / English</t>
         </is>
       </c>
     </row>
@@ -2209,17 +2165,17 @@
       <c r="A4" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="50" t="n">
+      <c r="B4" s="35" t="n">
         <v>46326</v>
       </c>
       <c r="C4" s="29" t="inlineStr">
         <is>
-          <t>Rotina de listening de 30 dias seguidos</t>
+          <t>30-day listening streak</t>
         </is>
       </c>
       <c r="D4" s="29" t="inlineStr">
         <is>
-          <t>Sequência de 30 dias na tarefa diária de listening.</t>
+          <t>30-day streak on the daily Listening task.</t>
         </is>
       </c>
     </row>
@@ -2227,17 +2183,17 @@
       <c r="A5" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="50" t="n">
+      <c r="B5" s="35" t="n">
         <v>46356</v>
       </c>
       <c r="C5" s="29" t="inlineStr">
         <is>
-          <t>Ler a documentação do pandas ("Getting started") sem tradutor</t>
+          <t>Read the pandas "Getting started" docs without a translator</t>
         </is>
       </c>
       <c r="D5" s="29" t="inlineStr">
         <is>
-          <t>Resumir em português, sem consultar tradução, o que cada seção ensina.</t>
+          <t>Summarize, without a translator, what each section teaches.</t>
         </is>
       </c>
     </row>
@@ -2245,17 +2201,17 @@
       <c r="A6" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="50" t="n">
+      <c r="B6" s="35" t="n">
         <v>46387</v>
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>Assistir a uma palestra técnica de 20 min com legenda em inglês</t>
+          <t>Watch a 20-minute tech talk with English subtitles</t>
         </is>
       </c>
       <c r="D6" s="29" t="inlineStr">
         <is>
-          <t>Resumo de 5 frases em inglês do que foi dito.</t>
+          <t>A 5-sentence summary in English of what was said.</t>
         </is>
       </c>
     </row>
@@ -2263,17 +2219,17 @@
       <c r="A7" s="34" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="50" t="n">
+      <c r="B7" s="35" t="n">
         <v>46418</v>
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>Escrever um README em inglês para um projeto seu</t>
+          <t>Write an English README for one of my projects</t>
         </is>
       </c>
       <c r="D7" s="29" t="inlineStr">
         <is>
-          <t>README publicado no GitHub, revisado pela IA.</t>
+          <t>README published on GitHub, reviewed by AI.</t>
         </is>
       </c>
     </row>
@@ -2281,17 +2237,17 @@
       <c r="A8" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="50" t="n">
+      <c r="B8" s="35" t="n">
         <v>46446</v>
       </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
-          <t>Ler um capítulo de uma fonte técnica em inglês sem tradutor</t>
+          <t>Explain a whole chapter out loud, in English, right after reading it</t>
         </is>
       </c>
       <c r="D8" s="29" t="inlineStr">
         <is>
-          <t>Cartão de revisão do capítulo escrito em inglês.</t>
+          <t>A 3-minute recording without notes.</t>
         </is>
       </c>
     </row>
@@ -2299,17 +2255,17 @@
       <c r="A9" s="34" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="50" t="n">
+      <c r="B9" s="35" t="n">
         <v>46477</v>
       </c>
       <c r="C9" s="29" t="inlineStr">
         <is>
-          <t>Palestra técnica de 30 min sem legenda</t>
+          <t>Watch a 30-minute tech talk without subtitles</t>
         </is>
       </c>
       <c r="D9" s="29" t="inlineStr">
         <is>
-          <t>Resumo falado de 2 minutos, gravado.</t>
+          <t>A 2-minute spoken summary, recorded.</t>
         </is>
       </c>
     </row>
@@ -2317,17 +2273,17 @@
       <c r="A10" s="34" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="50" t="n">
+      <c r="B10" s="35" t="n">
         <v>46507</v>
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
-          <t>Explicar um projeto seu em 5 minutos</t>
+          <t>Explain one of my projects in 5 minutes</t>
         </is>
       </c>
       <c r="D10" s="29" t="inlineStr">
         <is>
-          <t>Gravação sem roteiro lido.</t>
+          <t>A recording without reading a script.</t>
         </is>
       </c>
     </row>
@@ -2335,17 +2291,17 @@
       <c r="A11" s="34" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="50" t="n">
+      <c r="B11" s="35" t="n">
         <v>46538</v>
       </c>
       <c r="C11" s="29" t="inlineStr">
         <is>
-          <t>Escrever um post técnico de ~500 palavras</t>
+          <t>Write a ~500-word technical post</t>
         </is>
       </c>
       <c r="D11" s="29" t="inlineStr">
         <is>
-          <t>Post publicado (LinkedIn, blog ou GitHub).</t>
+          <t>Post published (LinkedIn, blog or GitHub).</t>
         </is>
       </c>
     </row>
@@ -2353,17 +2309,17 @@
       <c r="A12" s="34" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="50" t="n">
+      <c r="B12" s="35" t="n">
         <v>46568</v>
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
-          <t>Conversa de 20 min por voz com IA sobre um tema técnico</t>
+          <t>Hold a 20-minute voice conversation with AI on a technical topic</t>
         </is>
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>Conversa sem pausas longas nem troca para o português.</t>
+          <t>No long pauses and no switching to Portuguese.</t>
         </is>
       </c>
     </row>
@@ -2371,17 +2327,17 @@
       <c r="A13" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="50" t="n">
+      <c r="B13" s="35" t="n">
         <v>46599</v>
       </c>
       <c r="C13" s="29" t="inlineStr">
         <is>
-          <t>Simular uma reunião com cliente: apresentar uma proposta de projeto de dados</t>
+          <t>Simulate a client meeting: pitch a data project proposal</t>
         </is>
       </c>
       <c r="D13" s="29" t="inlineStr">
         <is>
-          <t>Gravação de 10 minutos.</t>
+          <t>A 10-minute recording.</t>
         </is>
       </c>
     </row>
@@ -2389,17 +2345,17 @@
       <c r="A14" s="34" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="50" t="n">
+      <c r="B14" s="35" t="n">
         <v>46630</v>
       </c>
       <c r="C14" s="29" t="inlineStr">
         <is>
-          <t>Participar de uma discussão técnica em inglês</t>
+          <t>Join a technical discussion in English</t>
         </is>
       </c>
       <c r="D14" s="29" t="inlineStr">
         <is>
-          <t>Uma issue ou pull request comentado em repositório público.</t>
+          <t>A comment on an issue or pull request in a public repository.</t>
         </is>
       </c>
     </row>
@@ -2407,17 +2363,17 @@
       <c r="A15" s="34" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="50" t="n">
+      <c r="B15" s="35" t="n">
         <v>46660</v>
       </c>
       <c r="C15" s="29" t="inlineStr">
         <is>
-          <t>Apresentar um case completo em inglês</t>
+          <t>Present a full case study in English</t>
         </is>
       </c>
       <c r="D15" s="29" t="inlineStr">
         <is>
-          <t>Apresentação de 10 minutos gravada.</t>
+          <t>A 10-minute recorded presentation.</t>
         </is>
       </c>
     </row>
@@ -2484,12 +2440,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Diagnóstico estatístico de vendas</t>
+          <t>Sales Statistical Diagnosis</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Estatística, SQL, Python</t>
+          <t>Statistics, SQL, Python</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -2497,7 +2453,7 @@
           <t>Relatório com consultas SQL e testes de hipótese (ex.: conversão de orçamentos em vendas por bloco).</t>
         </is>
       </c>
-      <c r="E4" s="51" t="n">
+      <c r="E4" s="36" t="n">
         <v>46387</v>
       </c>
     </row>
@@ -2509,12 +2465,12 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Análise de ruptura de estoque para a diretoria</t>
+          <t>Stockout Analysis for the Board</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>EDA avançada, matemática, visualização, storytelling</t>
+          <t>Advanced EDA, Mathematics, Data Visualization, Data Storytelling</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -2522,7 +2478,7 @@
           <t>EDA completa + apresentação de 10 slides com recomendação.</t>
         </is>
       </c>
-      <c r="E5" s="52" t="n">
+      <c r="E5" s="37" t="n">
         <v>46481</v>
       </c>
     </row>
@@ -2534,12 +2490,12 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Assistente de IA sobre a documentação das bases</t>
+          <t>AI Assistant for the Data Documentation (RAG)</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Engenharia de IA, engenharia de dados e governança, prompt</t>
+          <t>AI Engineering, Data Engineering and Governance, Prompt Engineering</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -2547,7 +2503,7 @@
           <t>App que responde perguntas sobre as bases a partir das descrições (RAG), com rotina de atualização.</t>
         </is>
       </c>
-      <c r="E6" s="53" t="n">
+      <c r="E6" s="38" t="n">
         <v>46572</v>
       </c>
     </row>
@@ -2559,12 +2515,12 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>Previsão de demanda ou ruptura em produção</t>
+          <t>Demand or Stockout Forecasting in Production</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>Engenharia de ML, system design</t>
+          <t>ML Engineering, System Design</t>
         </is>
       </c>
       <c r="D7" s="20" t="inlineStr">
@@ -2572,7 +2528,7 @@
           <t>Modelo treinado, servido e monitorado, com o desenho da arquitetura.</t>
         </is>
       </c>
-      <c r="E7" s="54" t="n">
+      <c r="E7" s="39" t="n">
         <v>46663</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Concept-led capabilities: learning focus field and focus-aware prompts
- New optional "Foco de aprendizagem" on a capability/project (text, JSON and
  FOCUS: import): the concept list and practice rules lead the order of the
  parts and the attached sources become references
- Project instructions, split-into-parts, study and review prompts adapt:
  best source per concept (or an exercise when no source covers it), no whole
  books, diagram-first practice, silent-bug hunting, DIAGRAM field on the card
- Capabilities plan and import file: the programming capability now lists the
  eight reference sources and its concept list and practice rules
- Document the concept-led mode

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JeoC1T6GvSfXrBZdTVZHj4
</commit_message>
<xml_diff>
--- a/planejamento/plano-capacidades.xlsx
+++ b/planejamento/plano-capacidades.xlsx
@@ -827,12 +827,12 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Book: Python for Data Analysis, 3rd ed. (Wes McKinney), free at wesmckinney.com/book</t>
+          <t>Book: Fundamentals of Data Engineering (Reis &amp; Housley)</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Repository: github.com/jakevdp/PythonDataScienceHandbook</t>
+          <t>Book: Designing Data-Intensive Applications (Kleppmann); Book: The Data Warehouse Toolkit (Kimball &amp; Ross); Book: A Philosophy of Software Design (Ousterhout); Book: How to Solve It (Pólya); Book: Data Pipelines Pocket Reference (Densmore); Book: Python Data Science Handbook (VanderPlas), free at jakevdp.github.io/PythonDataScienceHandbook; Site: c4model.com; Docs: Mermaid (mermaid.js.org)</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Ferramenta de tudo que vem depois; você já usa pandas, aqui fecha lacunas.</t>
+          <t>Guiada por conceitos, não por um livro: a lista de conceitos (campo Foco) manda na ordem e os livros são referências por conceito. Pensar e desenhar antes de pedir código à IA é o que mais multiplica o resto.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly plan for daily works and real-life practice for personal capabilities
- Daily works can hold a plan per weekday: the card shows today's title, the page
  shows today's full plan and the whole week, editable by the owner
- Personal-area capabilities get prompts with real-life experiments and scenes
  instead of datasets and scripts, and a fair stance on religious books
- Plan files: personal capabilities (three books) in the spreadsheet and as an
  import file; routine notes updated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JeoC1T6GvSfXrBZdTVZHj4
</commit_message>
<xml_diff>
--- a/planejamento/plano-capacidades.xlsx
+++ b/planejamento/plano-capacidades.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Rotina semanal" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Inglês — marcos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Projetos integradores" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Capacidades pessoais" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Capacidades'!$A$4:$M$19</definedName>
@@ -130,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -238,6 +239,15 @@
     </xf>
     <xf numFmtId="165" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1791,7 +1801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2109,6 +2119,20 @@
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Capacidade semanal estimada: 10 sessões nas noites úteis + 12 no fim de semana = 22 (aba Premissas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Leitura pessoal: 2 sessões no domingo à tarde, a partir de 06/11/2026 (aba Capacidades pessoais). Elas saem das 22 sessões por semana depois que Git termina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Exercício (calistenia) e caminhada de domingo: ficam nas tarefas diárias, com o plano da semana em Exercício físico.</t>
         </is>
       </c>
     </row>
@@ -2542,4 +2566,264 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="56" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Capacidades pessoais (leitura com aplicação na vida real)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Azul = valores para você ajustar. 2 sessões por semana, no domingo à tarde. Uma de cada vez; a próxima começa quando a anterior termina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Ordem</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Capacidade</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Área</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Profundidade</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Partes estimadas</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Sessões por semana</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Início</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Semanas estimadas</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Prazo estimado</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Por que nesta posição</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Prática</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>How to Win Friends and Influence People</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>Pessoal</t>
+        </is>
+      </c>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>Sólido</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="F5" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="41" t="n">
+        <v>46332</v>
+      </c>
+      <c r="H5" s="34">
+        <f>ROUNDUP(E5*IF(D5="Profundo",Premissas!$B$4,Premissas!$B$5)/F5,0)</f>
+        <v/>
+      </c>
+      <c r="I5" s="42">
+        <f>G5+H5*7</f>
+        <v/>
+      </c>
+      <c r="J5" s="29" t="inlineStr">
+        <is>
+          <t>Book: How to Win Friends and Influence People (Dale Carnegie), Portuguese edition: Como Fazer Amigos e Influenciar Pessoas</t>
+        </is>
+      </c>
+      <c r="K5" s="29" t="inlineStr">
+        <is>
+          <t>Capítulos curtos e práticos, com retorno imediato no trabalho com clientes e na vida pessoal. Começa quando Git termina e libera 3 sessões por semana.</t>
+        </is>
+      </c>
+      <c r="L5" s="29" t="inlineStr">
+        <is>
+          <t>Um princípio por semana vira um experimento em conversas reais (trabalho, família, clientes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>The 7 Habits of Highly Effective People</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>Pessoal</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>Sólido</t>
+        </is>
+      </c>
+      <c r="E6" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="F6" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="41" t="n">
+        <v>46419</v>
+      </c>
+      <c r="H6" s="34">
+        <f>ROUNDUP(E6*IF(D6="Profundo",Premissas!$B$4,Premissas!$B$5)/F6,0)</f>
+        <v/>
+      </c>
+      <c r="I6" s="42">
+        <f>G6+H6*7</f>
+        <v/>
+      </c>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>Book: The 7 Habits of Highly Effective People (Stephen R. Covey), Portuguese edition: Os 7 Hábitos das Pessoas Altamente Eficazes</t>
+        </is>
+      </c>
+      <c r="K6" s="29" t="inlineStr">
+        <is>
+          <t>É cumulativo (vitória privada, depois pública) e conversa com o projeto de disciplina. Vem depois de Carnegie, que prepara os hábitos 4 a 6.</t>
+        </is>
+      </c>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t>Um hábito vira uma regra pessoal de 7 dias, anotada no app como tarefa diária.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>Mere Christianity</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Pessoal</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>Conceitual</t>
+        </is>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="41" t="n">
+        <v>46489</v>
+      </c>
+      <c r="H7" s="34">
+        <f>ROUNDUP(E7*IF(D7="Profundo",Premissas!$B$4,Premissas!$B$5)/F7,0)</f>
+        <v/>
+      </c>
+      <c r="I7" s="42">
+        <f>G7+H7*7</f>
+        <v/>
+      </c>
+      <c r="J7" s="29" t="inlineStr">
+        <is>
+          <t>Book: Mere Christianity (C. S. Lewis), Portuguese edition: Cristianismo Puro e Simples</t>
+        </is>
+      </c>
+      <c r="K7" s="29" t="inlineStr">
+        <is>
+          <t>É o mais longo e o menos urgente; lê-se melhor com calma, aos domingos. Pode ir para o início se for prioridade para você.</t>
+        </is>
+      </c>
+      <c r="L7" s="29" t="inlineStr">
+        <is>
+          <t>Cada parte termina com uma pergunta para refletir ou conversar; sem dados, sem scripts.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Day guide, practice rules, Git folded into programming, reminders file
- Home shows a "Guia do dia": ordered steps by time block (daily works, study
  sessions picked from active capabilities, due reviews, pre-reading), checkable,
  with adjustable times and number of sessions; daily works get a "when" block
- New "Regras de prática" field: practice rules without changing the part order
  (prompts, import, JSON); SQL uses it, programming keeps its concept focus
- Plan files: Git becomes a track of the programming capability, SQL owns data
  modeling, personal reading dates and notes updated
- planejamento/lembretes-foco.ics: daily morning and evening reminders

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JeoC1T6GvSfXrBZdTVZHj4
</commit_message>
<xml_diff>
--- a/planejamento/plano-capacidades.xlsx
+++ b/planejamento/plano-capacidades.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Capacidades pessoais" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Capacidades'!$A$4:$M$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Capacidades'!$A$4:$M$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -331,17 +331,17 @@
     <author>Plano</author>
   </authors>
   <commentList>
-    <comment ref="E19" authorId="0" shapeId="0">
+    <comment ref="E18" authorId="0" shapeId="0">
       <text>
         <t>12 marcos mensais, um por parte.</t>
       </text>
     </comment>
-    <comment ref="F19" authorId="0" shapeId="0">
+    <comment ref="F18" authorId="0" shapeId="0">
       <text>
         <t>1 sessão no fim de semana para o marco; o resto é o hábito diário do almoço.</t>
       </text>
     </comment>
-    <comment ref="H19" authorId="0" shapeId="0">
+    <comment ref="H18" authorId="0" shapeId="0">
       <text>
         <t>Contínua: o ano inteiro, sem fórmula.</t>
       </text>
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>5</v>
@@ -842,7 +842,7 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Book: Designing Data-Intensive Applications (Kleppmann); Book: The Data Warehouse Toolkit (Kimball &amp; Ross); Book: A Philosophy of Software Design (Ousterhout); Book: How to Solve It (Pólya); Book: Data Pipelines Pocket Reference (Densmore); Book: Python Data Science Handbook (VanderPlas), free at jakevdp.github.io/PythonDataScienceHandbook; Site: c4model.com; Docs: Mermaid (mermaid.js.org)</t>
+          <t>Book: Designing Data-Intensive Applications (Kleppmann); Book: The Data Warehouse Toolkit (Kimball &amp; Ross); Book: A Philosophy of Software Design (Ousterhout); Book: How to Solve It (Pólya); Book: Data Pipelines Pocket Reference (Densmore); Book: Python Data Science Handbook (VanderPlas), free at jakevdp.github.io/PythonDataScienceHandbook; Book: Pro Git, 2nd ed. (Chacon &amp; Straub), free at git-scm.com/book — chapters 1–3 and 10 (the Git track); Site: c4model.com; Docs: Mermaid (mermaid.js.org)</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Guiada por conceitos, não por um livro: a lista de conceitos (campo Foco) manda na ordem e os livros são referências por conceito. Pensar e desenhar antes de pedir código à IA é o que mais multiplica o resto.</t>
+          <t>Guiada por conceitos, não por um livro: a lista de conceitos (campo Foco) manda na ordem e os livros são referências. Inclui a trilha de Git (cerca de 8 partes). Pensar e desenhar antes de pedir código à IA é o que mais multiplica o resto.</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>A linguagem dos dados em qualquer empresa cliente.</t>
+          <t>A linguagem dos dados em qualquer empresa cliente. É dona da modelagem de dados (granularidade, chaves, esquema em estrela); as regras de prática vêm do campo Regras de prática.</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Git (Conceptual)</t>
+          <t>Prompt Engineering / Harness / Spec</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -933,17 +933,17 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Conceitual</t>
+          <t>Sólido</t>
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>46296</v>
+        <v>46332</v>
       </c>
       <c r="H8" s="4">
         <f>ROUNDUP(E8*IF(D8="Profundo",Premissas!$B$4,Premissas!$B$5)/F8,0)</f>
@@ -955,81 +955,81 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Book: Pro Git, 2nd ed. (Chacon &amp; Straub), free at git-scm.com/book — chapters 1–3 and 10</t>
+          <t>Repository: github.com/anthropics/prompt-eng-interactive-tutorial</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Article: Building effective agents (Anthropic); Docs: Anthropic documentation on prompting and agents</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Começa em 06/11/2026</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Curta; base para versionar projetos e montar portfólio.</t>
+          <t>Multiplica o seu método de estudo com IA e já vira serviço.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Prompt Engineering / Harness / Spec</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics for Data Science</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Profissional</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Sólido</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>46332</v>
-      </c>
-      <c r="H9" s="4">
+      <c r="E9" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>46391</v>
+      </c>
+      <c r="H9" s="9">
         <f>ROUNDUP(E9*IF(D9="Profundo",Premissas!$B$4,Premissas!$B$5)/F9,0)</f>
         <v/>
       </c>
-      <c r="I9" s="8">
+      <c r="I9" s="13">
         <f>G9+H9*7</f>
         <v/>
       </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Repository: github.com/anthropics/prompt-eng-interactive-tutorial</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>Article: Building effective agents (Anthropic); Docs: Anthropic documentation on prompting and agents</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>Começa quando Git termina</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>Multiplica o seu método de estudo com IA e já vira serviço.</t>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>Book: Mathematics for Machine Learning (Deisenroth, Faisal &amp; Ong), free at mml-book.github.io</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>Course: Essence of Linear Algebra (3Blue1Brown)</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Statistics for Data Science</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>Destrava ML: álgebra linear, cálculo e otimização aplicados.</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Mathematics for Data Science</t>
+          <t>Advanced EDA</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -1051,14 +1051,14 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Sólido</t>
+          <t>Profundo</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G10" s="12" t="n">
         <v>46391</v>
@@ -1073,22 +1073,22 @@
       </c>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>Book: Mathematics for Machine Learning (Deisenroth, Faisal &amp; Ong), free at mml-book.github.io</t>
+          <t>Book: Feature Engineering and Selection (Kuhn &amp; Johnson), free at feat.engineering</t>
         </is>
       </c>
       <c r="K10" s="10" t="inlineStr">
         <is>
-          <t>Course: Essence of Linear Algebra (3Blue1Brown)</t>
+          <t>Repository: github.com/jakevdp/PythonDataScienceHandbook; My own datasets</t>
         </is>
       </c>
       <c r="L10" s="10" t="inlineStr">
         <is>
-          <t>Statistics for Data Science</t>
+          <t>Statistics; Python for Data Science</t>
         </is>
       </c>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t>Destrava ML: álgebra linear, cálculo e otimização aplicados.</t>
+          <t>Onde você gera valor mais rápido para um cliente.</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Advanced EDA</t>
+          <t>Data Visualization</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -1110,14 +1110,14 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Profundo</t>
+          <t>Sólido</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G11" s="12" t="n">
         <v>46391</v>
@@ -1132,22 +1132,22 @@
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>Book: Feature Engineering and Selection (Kuhn &amp; Johnson), free at feat.engineering</t>
+          <t>Book: Fundamentals of Data Visualization (Claus Wilke), free at clauswilke.com/dataviz</t>
         </is>
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>Repository: github.com/jakevdp/PythonDataScienceHandbook; My own datasets</t>
+          <t>Docs: matplotlib and seaborn</t>
         </is>
       </c>
       <c r="L11" s="10" t="inlineStr">
         <is>
-          <t>Statistics; Python for Data Science</t>
+          <t>Python for Data Science</t>
         </is>
       </c>
       <c r="M11" s="10" t="inlineStr">
         <is>
-          <t>Onde você gera valor mais rápido para um cliente.</t>
+          <t>Base para comunicar qualquer análise.</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Data Visualization</t>
+          <t>Data Storytelling</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -1173,13 +1173,13 @@
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>46391</v>
+        <v>46447</v>
       </c>
       <c r="H12" s="9">
         <f>ROUNDUP(E12*IF(D12="Profundo",Premissas!$B$4,Premissas!$B$5)/F12,0)</f>
@@ -1191,81 +1191,81 @@
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>Book: Fundamentals of Data Visualization (Claus Wilke), free at clauswilke.com/dataviz</t>
+          <t>Book: Storytelling with Data (Cole Nussbaumer Knaflic)</t>
         </is>
       </c>
       <c r="K12" s="10" t="inlineStr">
         <is>
-          <t>Docs: matplotlib and seaborn</t>
+          <t>Book: Storytelling with Data: Let's Practice! (Knaflic)</t>
         </is>
       </c>
       <c r="L12" s="10" t="inlineStr">
         <is>
-          <t>Python for Data Science</t>
+          <t>Data Visualization</t>
         </is>
       </c>
       <c r="M12" s="10" t="inlineStr">
         <is>
-          <t>Base para comunicar qualquer análise.</t>
+          <t>Explicar e vender o resultado é metade da consultoria.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Data Storytelling</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>AI Engineering</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>Profissional</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>Sólido</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="F13" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" s="12" t="n">
-        <v>46447</v>
-      </c>
-      <c r="H13" s="9">
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Profundo</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>46482</v>
+      </c>
+      <c r="H13" s="14">
         <f>ROUNDUP(E13*IF(D13="Profundo",Premissas!$B$4,Premissas!$B$5)/F13,0)</f>
         <v/>
       </c>
-      <c r="I13" s="13">
+      <c r="I13" s="18">
         <f>G13+H13*7</f>
         <v/>
       </c>
-      <c r="J13" s="10" t="inlineStr">
-        <is>
-          <t>Book: Storytelling with Data (Cole Nussbaumer Knaflic)</t>
-        </is>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>Book: Storytelling with Data: Let's Practice! (Knaflic)</t>
-        </is>
-      </c>
-      <c r="L13" s="10" t="inlineStr">
-        <is>
-          <t>Data Visualization</t>
-        </is>
-      </c>
-      <c r="M13" s="10" t="inlineStr">
-        <is>
-          <t>Explicar e vender o resultado é metade da consultoria.</t>
+      <c r="J13" s="15" t="inlineStr">
+        <is>
+          <t>Book: AI Engineering (Chip Huyen)</t>
+        </is>
+      </c>
+      <c r="K13" s="15" t="inlineStr">
+        <is>
+          <t>Article: Building effective agents (Anthropic)</t>
+        </is>
+      </c>
+      <c r="L13" s="15" t="inlineStr">
+        <is>
+          <t>Prompt Engineering / Harness / Spec; Python</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>Aplicações com LLM: o serviço mais demandado agora.</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>AI Engineering</t>
+          <t>Data Engineering and Governance</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -1287,14 +1287,14 @@
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>Profundo</t>
+          <t>Sólido</t>
         </is>
       </c>
       <c r="E14" s="16" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G14" s="17" t="n">
         <v>46482</v>
@@ -1309,22 +1309,22 @@
       </c>
       <c r="J14" s="15" t="inlineStr">
         <is>
-          <t>Book: AI Engineering (Chip Huyen)</t>
+          <t>Book: Fundamentals of Data Engineering (Reis &amp; Housley)</t>
         </is>
       </c>
       <c r="K14" s="15" t="inlineStr">
         <is>
-          <t>Article: Building effective agents (Anthropic)</t>
+          <t>Repository: github.com/DataTalksClub/data-engineering-zoomcamp; Book: Data Governance: The Definitive Guide (Eryurek et al.)</t>
         </is>
       </c>
       <c r="L14" s="15" t="inlineStr">
         <is>
-          <t>Prompt Engineering / Harness / Spec; Python</t>
+          <t>SQL / Data Modeling; Python</t>
         </is>
       </c>
       <c r="M14" s="15" t="inlineStr">
         <is>
-          <t>Aplicações com LLM: o serviço mais demandado agora.</t>
+          <t>Sem dados confiáveis nenhum projeto de cliente fica de pé.</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>Data Engineering and Governance</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
@@ -1346,14 +1346,14 @@
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>Sólido</t>
+          <t>Conceitual</t>
         </is>
       </c>
       <c r="E15" s="16" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G15" s="17" t="n">
         <v>46482</v>
@@ -1368,81 +1368,81 @@
       </c>
       <c r="J15" s="15" t="inlineStr">
         <is>
-          <t>Book: Fundamentals of Data Engineering (Reis &amp; Housley)</t>
+          <t>Book: Grokking Algorithms, 2nd ed. (Aditya Bhargava)</t>
         </is>
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>Repository: github.com/DataTalksClub/data-engineering-zoomcamp; Book: Data Governance: The Definitive Guide (Eryurek et al.)</t>
+          <t>Course: CS50x (Harvard, free)</t>
         </is>
       </c>
       <c r="L15" s="15" t="inlineStr">
         <is>
-          <t>SQL / Data Modeling; Python</t>
+          <t>Programming Logic</t>
         </is>
       </c>
       <c r="M15" s="15" t="inlineStr">
         <is>
-          <t>Sem dados confiáveis nenhum projeto de cliente fica de pé.</t>
+          <t>Estruturas de dados e complexidade para código que escala.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>Computer Science</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>ML Engineering</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>Profissional</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>Conceitual</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="F16" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <v>46482</v>
-      </c>
-      <c r="H16" s="14">
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>Profundo</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="F16" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" s="22" t="n">
+        <v>46573</v>
+      </c>
+      <c r="H16" s="19">
         <f>ROUNDUP(E16*IF(D16="Profundo",Premissas!$B$4,Premissas!$B$5)/F16,0)</f>
         <v/>
       </c>
-      <c r="I16" s="18">
+      <c r="I16" s="23">
         <f>G16+H16*7</f>
         <v/>
       </c>
-      <c r="J16" s="15" t="inlineStr">
-        <is>
-          <t>Book: Grokking Algorithms, 2nd ed. (Aditya Bhargava)</t>
-        </is>
-      </c>
-      <c r="K16" s="15" t="inlineStr">
-        <is>
-          <t>Course: CS50x (Harvard, free)</t>
-        </is>
-      </c>
-      <c r="L16" s="15" t="inlineStr">
-        <is>
-          <t>Programming Logic</t>
-        </is>
-      </c>
-      <c r="M16" s="15" t="inlineStr">
-        <is>
-          <t>Estruturas de dados e complexidade para código que escala.</t>
+      <c r="J16" s="20" t="inlineStr">
+        <is>
+          <t>Book: Designing Machine Learning Systems (Chip Huyen)</t>
+        </is>
+      </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>Repository: github.com/GokuMohandas/Made-With-ML; Book: Hands-On Machine Learning (Aurélien Géron)</t>
+        </is>
+      </c>
+      <c r="L16" s="20" t="inlineStr">
+        <is>
+          <t>Mathematics; Statistics; Advanced EDA</t>
+        </is>
+      </c>
+      <c r="M16" s="20" t="inlineStr">
+        <is>
+          <t>Modelos em produção, do dado ao monitoramento.</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>ML Engineering</t>
+          <t>System Design</t>
         </is>
       </c>
       <c r="C17" s="20" t="inlineStr">
@@ -1464,14 +1464,14 @@
       </c>
       <c r="D17" s="20" t="inlineStr">
         <is>
-          <t>Profundo</t>
+          <t>Sólido</t>
         </is>
       </c>
       <c r="E17" s="21" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="F17" s="21" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G17" s="22" t="n">
         <v>46573</v>
@@ -1486,150 +1486,91 @@
       </c>
       <c r="J17" s="20" t="inlineStr">
         <is>
-          <t>Book: Designing Machine Learning Systems (Chip Huyen)</t>
+          <t>Book: Designing Data-Intensive Applications (Martin Kleppmann)</t>
         </is>
       </c>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Repository: github.com/GokuMohandas/Made-With-ML; Book: Hands-On Machine Learning (Aurélien Géron)</t>
+          <t>Repository: github.com/donnemartin/system-design-primer</t>
         </is>
       </c>
       <c r="L17" s="20" t="inlineStr">
         <is>
-          <t>Mathematics; Statistics; Advanced EDA</t>
+          <t>Data Engineering; AI Engineering</t>
         </is>
       </c>
       <c r="M17" s="20" t="inlineStr">
         <is>
-          <t>Modelos em produção, do dado ao monitoramento.</t>
+          <t>Desenhar a solução inteira para o cliente.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>System Design</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>Contínua</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="inlineStr">
         <is>
           <t>Profissional</t>
         </is>
       </c>
-      <c r="D18" s="20" t="inlineStr">
+      <c r="D18" s="25" t="inlineStr">
         <is>
           <t>Sólido</t>
         </is>
       </c>
-      <c r="E18" s="21" t="n">
-        <v>30</v>
-      </c>
-      <c r="F18" s="21" t="n">
-        <v>6</v>
-      </c>
-      <c r="G18" s="22" t="n">
-        <v>46573</v>
-      </c>
-      <c r="H18" s="19">
-        <f>ROUNDUP(E18*IF(D18="Profundo",Premissas!$B$4,Premissas!$B$5)/F18,0)</f>
-        <v/>
-      </c>
-      <c r="I18" s="23">
-        <f>G18+H18*7</f>
-        <v/>
-      </c>
-      <c r="J18" s="20" t="inlineStr">
-        <is>
-          <t>Book: Designing Data-Intensive Applications (Martin Kleppmann)</t>
-        </is>
-      </c>
-      <c r="K18" s="20" t="inlineStr">
-        <is>
-          <t>Repository: github.com/donnemartin/system-design-primer</t>
-        </is>
-      </c>
-      <c r="L18" s="20" t="inlineStr">
-        <is>
-          <t>Data Engineering; AI Engineering</t>
-        </is>
-      </c>
-      <c r="M18" s="20" t="inlineStr">
-        <is>
-          <t>Desenhar a solução inteira para o cliente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="24" t="inlineStr">
-        <is>
-          <t>Contínua</t>
-        </is>
-      </c>
-      <c r="B19" s="25" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="C19" s="25" t="inlineStr">
-        <is>
-          <t>Profissional</t>
-        </is>
-      </c>
-      <c r="D19" s="25" t="inlineStr">
-        <is>
-          <t>Sólido</t>
-        </is>
-      </c>
-      <c r="E19" s="26" t="n">
+      <c r="E18" s="26" t="n">
         <v>12</v>
       </c>
-      <c r="F19" s="26" t="n">
+      <c r="F18" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="27" t="n">
+      <c r="G18" s="27" t="n">
         <v>46296</v>
       </c>
-      <c r="H19" s="26" t="n">
+      <c r="H18" s="26" t="n">
         <v>52</v>
       </c>
-      <c r="I19" s="27" t="n">
+      <c r="I18" s="27" t="n">
         <v>46660</v>
       </c>
-      <c r="J19" s="25" t="inlineStr">
+      <c r="J18" s="25" t="inlineStr">
         <is>
           <t>Book: English Grammar in Use (Raymond Murphy) — grammar topics only</t>
         </is>
       </c>
-      <c r="K19" s="25" t="inlineStr">
+      <c r="K18" s="25" t="inlineStr">
         <is>
           <t>Tech talks (PyData, conferences); The sources of every other capability, all studied in English</t>
         </is>
       </c>
-      <c r="L19" s="25" t="inlineStr">
+      <c r="L18" s="25" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M19" s="25" t="inlineStr">
+      <c r="M18" s="25" t="inlineStr">
         <is>
           <t>Habilidade, não conceito: 12 marcos mensais (aba Inglês — marcos) + hábito diário no almoço + todas as capacidades estudadas em inglês (imersão diária).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Fontes: sugestões em inglês (o estudo das capacidades é em inglês); troque à vontade. A primeira fonte é a que define a ordem das partes.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M19"/>
+  <autoFilter ref="A4:M18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -1772,7 +1713,7 @@
     <row r="13">
       <c r="A13" s="33" t="inlineStr">
         <is>
-          <t>• Não estude as 15 capacidades em paralelo: 1 profunda + 1 ou 2 sólidas + às vezes 1 curta por vez.</t>
+          <t>• Não estude as 14 capacidades em paralelo: 1 profunda + 1 ou 2 sólidas + às vezes 1 curta por vez.</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2066,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Leitura pessoal: 2 sessões no domingo à tarde, a partir de 06/11/2026 (aba Capacidades pessoais). Elas saem das 22 sessões por semana depois que Git termina.</t>
+          <t>Leitura pessoal: 2 sessões no domingo à tarde, a partir de 06/11/2026 (aba Capacidades pessoais). Entram nas 22 sessões por semana; de novembro a 03/12 a carga fica cerca de 1 sessão acima, e isso some quando Programação e SQL terminam.</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2651,7 @@
       </c>
       <c r="K5" s="29" t="inlineStr">
         <is>
-          <t>Capítulos curtos e práticos, com retorno imediato no trabalho com clientes e na vida pessoal. Começa quando Git termina e libera 3 sessões por semana.</t>
+          <t>Capítulos curtos e práticos, com retorno imediato no trabalho com clientes e na vida pessoal. Começa em 06/11/2026.</t>
         </is>
       </c>
       <c r="L5" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Personal plan: run Carnegie and Lewis in parallel, Covey after
One session per week each (Saturday and Sunday); dates and notes updated in the
spreadsheet and the personal import file.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JeoC1T6GvSfXrBZdTVZHj4
</commit_message>
<xml_diff>
--- a/planejamento/plano-capacidades.xlsx
+++ b/planejamento/plano-capacidades.xlsx
@@ -2066,7 +2066,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Leitura pessoal: 2 sessões no domingo à tarde, a partir de 06/11/2026 (aba Capacidades pessoais). Entram nas 22 sessões por semana; de novembro a 03/12 a carga fica cerca de 1 sessão acima, e isso some quando Programação e SQL terminam.</t>
+          <t>Leitura pessoal: 2 sessões por semana, Carnegie no sábado e Lewis no domingo, a partir de 06/11/2026 (aba Capacidades pessoais). Entram nas 22 sessões por semana; de novembro a 03/12 a carga fica cerca de 1 sessão acima, e isso some quando Programação e SQL terminam.</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2542,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Azul = valores para você ajustar. 2 sessões por semana, no domingo à tarde. Uma de cada vez; a próxima começa quando a anterior termina.</t>
+          <t>Azul = valores para você ajustar. 1 sessão por semana em cada livro: Carnegie no sábado e Lewis no domingo, juntos. Covey começa quando Lewis termina.</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
         <v>20</v>
       </c>
       <c r="F5" s="40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" s="41" t="n">
         <v>46332</v>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="K5" s="29" t="inlineStr">
         <is>
-          <t>Capítulos curtos e práticos, com retorno imediato no trabalho com clientes e na vida pessoal. Começa em 06/11/2026.</t>
+          <t>Roda junto com Mere Christianity, 1 sessão por semana, no sábado. Uma sessão por semana combina com os experimentos de 3 a 7 dias.</t>
         </is>
       </c>
       <c r="L5" s="29" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>The 7 Habits of Highly Effective People</t>
+          <t>Mere Christianity</t>
         </is>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -2676,17 +2676,17 @@
       </c>
       <c r="D6" s="29" t="inlineStr">
         <is>
-          <t>Sólido</t>
+          <t>Conceitual</t>
         </is>
       </c>
       <c r="E6" s="40" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="41" t="n">
-        <v>46419</v>
+        <v>46332</v>
       </c>
       <c r="H6" s="34">
         <f>ROUNDUP(E6*IF(D6="Profundo",Premissas!$B$4,Premissas!$B$5)/F6,0)</f>
@@ -2698,17 +2698,17 @@
       </c>
       <c r="J6" s="29" t="inlineStr">
         <is>
-          <t>Book: The 7 Habits of Highly Effective People (Stephen R. Covey), Portuguese edition: Os 7 Hábitos das Pessoas Altamente Eficazes</t>
+          <t>Book: Mere Christianity (C. S. Lewis), Portuguese edition: Cristianismo Puro e Simples</t>
         </is>
       </c>
       <c r="K6" s="29" t="inlineStr">
         <is>
-          <t>É cumulativo (vitória privada, depois pública) e conversa com o projeto de disciplina. Vem depois de Carnegie, que prepara os hábitos 4 a 6.</t>
+          <t>Roda junto com Carnegie, 1 sessão por semana, no domingo. É um argumento para ler com calma e termina primeiro.</t>
         </is>
       </c>
       <c r="L6" s="29" t="inlineStr">
         <is>
-          <t>Um hábito vira uma regra pessoal de 7 dias, anotada no app como tarefa diária.</t>
+          <t>Cada parte termina com uma pergunta para refletir ou conversar; sem dados, sem scripts.</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t>Mere Christianity</t>
+          <t>The 7 Habits of Highly Effective People</t>
         </is>
       </c>
       <c r="C7" s="29" t="inlineStr">
@@ -2728,17 +2728,17 @@
       </c>
       <c r="D7" s="29" t="inlineStr">
         <is>
-          <t>Conceitual</t>
+          <t>Sólido</t>
         </is>
       </c>
       <c r="E7" s="40" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" s="41" t="n">
-        <v>46489</v>
+        <v>46458</v>
       </c>
       <c r="H7" s="34">
         <f>ROUNDUP(E7*IF(D7="Profundo",Premissas!$B$4,Premissas!$B$5)/F7,0)</f>
@@ -2750,17 +2750,17 @@
       </c>
       <c r="J7" s="29" t="inlineStr">
         <is>
-          <t>Book: Mere Christianity (C. S. Lewis), Portuguese edition: Cristianismo Puro e Simples</t>
+          <t>Book: The 7 Habits of Highly Effective People (Stephen R. Covey), Portuguese edition: Os 7 Hábitos das Pessoas Altamente Eficazes</t>
         </is>
       </c>
       <c r="K7" s="29" t="inlineStr">
         <is>
-          <t>É o mais longo e o menos urgente; lê-se melhor com calma, aos domingos. Pode ir para o início se for prioridade para você.</t>
+          <t>Começa quando Mere Christianity termina, com 1 sessão por semana. Quando Carnegie terminar (23/04/2027), suba para 2 sessões por semana.</t>
         </is>
       </c>
       <c r="L7" s="29" t="inlineStr">
         <is>
-          <t>Cada parte termina com uma pergunta para refletir ou conversar; sem dados, sem scripts.</t>
+          <t>Um hábito vira uma regra pessoal de 7 dias, anotada no app como tarefa diária.</t>
         </is>
       </c>
     </row>

</xml_diff>